<commit_message>
Fix issues preventing users from completing the budget guide wizard
Corrected a validation schema error in `schema.ts` to include "philanthropy" and added default values for `schoolProfile` in `public-wizard/index.tsx`, resolving navigation blockers in the budgeting wizard.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 87b038bd-f63c-42f8-9fe4-de4ac774b0a1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/XSlVKzA
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -155,7 +155,7 @@
     <t>CSP Startup Grant</t>
   </si>
   <si>
-    <t>Grants &amp; Contributions</t>
+    <t>Philanthropy</t>
   </si>
   <si>
     <t>Annual Fixed</t>
@@ -690,7 +690,7 @@
     <font>
       <i/>
       <color rgb="FF666666"/>
-      <sz val="10"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -706,7 +706,7 @@
     <font>
       <i/>
       <color rgb="FF888888"/>
-      <sz val="10"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -718,7 +718,7 @@
     <font>
       <i/>
       <color rgb="FF9CA3AF"/>
-      <sz val="9"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>

</xml_diff>

<commit_message>
Update application text and remove em dashes from various files
Replace em dashes (—) with standard dashes (-) and adjust wording across multiple files, including TypeScript, Excel exports, and markdown documentation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 267a4ab1-1bc3-48c3-827a-4ebff5905e8b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/69P15m5
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="213">
   <si>
-    <t>Heritage Academy Charter — Financial Model Assumptions</t>
+    <t>Heritage Academy Charter - Financial Model Assumptions</t>
   </si>
   <si>
     <t>Yellow cells are editable inputs. All other cells in this workbook are formulas.</t>
@@ -404,7 +404,7 @@
     <t>Built by SchoolStack Budget  •  budget.schoolstack.ai</t>
   </si>
   <si>
-    <t>Heritage Academy Charter — 5-Year Financial Model</t>
+    <t>Heritage Academy Charter - 5-Year Financial Model</t>
   </si>
   <si>
     <t>REVENUE</t>
@@ -575,7 +575,7 @@
     <t>Break-Even Enrollment</t>
   </si>
   <si>
-    <t>Heritage Academy Charter — 2026-27 Pro Forma</t>
+    <t>Heritage Academy Charter - 2026-27 Pro Forma</t>
   </si>
   <si>
     <t>August</t>

</xml_diff>

<commit_message>
Task #102: Financial Health dashboard tab across all 5 Excel exports
- Added break-even indicator rows to P&L tabs in all 5 export formats:
  formula-export.ts, lender-proforma-export.ts (also added cumulative NI),
  excel-export.ts, underwriting-export.ts, underwriting-workbook.ts
- Fixed DASHBOARD_GREEN import in formula-export.ts, underwriting-export.ts,
  underwriting-workbook.ts, and lender-proforma-export.ts
- Added revenueCategories to addDashboardSheet calls in all 4 exports that
  were missing it (formula, lender, underwriting v1, underwriting v2) so
  Revenue Sources metric shows accurate category counts
- Enhanced QA tests with runDashboardTieOuts: verifies 7 metric labels
  (Payroll %, Facility %, Operating Margin, DSCR, Revenue per Student,
  Revenue Sources, Break-even) and Benchmark column presence
- All QA suites pass: 24/24 exports, 33/33 parity, 3/3 formula-results
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -15,7 +15,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Instructions'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Assumptions'!$A1:$J80</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Assumptions'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'5-Year Model'!$A1:$F84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'5-Year Model'!$A1:$F85</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'5-Year Model'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Year 1 Pro Forma'!$A1:$N54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Year 1 Pro Forma'!$1:$2</definedName>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="306">
   <si>
     <t>How to Use This Workbook</t>
   </si>
@@ -606,6 +606,12 @@
   </si>
   <si>
     <t>Cumulative Net Income</t>
+  </si>
+  <si>
+    <t>Break-even</t>
+  </si>
+  <si>
+    <t>✓ Break-even</t>
   </si>
   <si>
     <t>CASH FLOW &amp; DEBT COVERAGE</t>
@@ -1040,14 +1046,14 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <i/>
-      <color rgb="FF6B7280"/>
+      <b/>
+      <color rgb="FF16A34A"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF16A34A"/>
+      <i/>
+      <color rgb="FF6B7280"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -1152,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1197,13 +1203,19 @@
     <xf numFmtId="165" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1227,27 +1239,24 @@
     <xf numFmtId="165" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="12" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="12" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3118,7 +3127,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -4135,500 +4144,520 @@
         <v>6668055</v>
       </c>
     </row>
-    <row r="60" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="12" t="s">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="30" t="s">
         <v>193</v>
       </c>
-      <c r="B60" s="12"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="12"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="27" t="s">
+      <c r="B59" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="B61" s="31">
+      <c r="D59" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="E59" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="F59" s="36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="B61" s="12"/>
+      <c r="C61" s="12"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="12"/>
+      <c r="F61" s="12"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="B62" s="31">
         <f>B50-B51-B52</f>
         <v>-105535</v>
       </c>
-      <c r="C61" s="31">
+      <c r="C62" s="31">
         <f>C50-C51-C52</f>
         <v>501148</v>
       </c>
-      <c r="D61" s="31">
+      <c r="D62" s="31">
         <f>D50-D51-D52</f>
         <v>1334490</v>
       </c>
-      <c r="E61" s="31">
+      <c r="E62" s="31">
         <f>E50-E51-E52</f>
         <v>2179988</v>
       </c>
-      <c r="F61" s="31">
+      <c r="F62" s="31">
         <f>F50-F51-F52</f>
         <v>3116109</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="B62" s="21">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="B63" s="21">
         <f>B53</f>
         <v>106629</v>
       </c>
-      <c r="C62" s="21">
+      <c r="C63" s="21">
         <f>C53</f>
         <v>66629</v>
       </c>
-      <c r="D62" s="21">
+      <c r="D63" s="21">
         <f>D53</f>
         <v>71629</v>
       </c>
-      <c r="E62" s="21">
+      <c r="E63" s="21">
         <f>E53</f>
         <v>56629</v>
       </c>
-      <c r="F62" s="21">
+      <c r="F63" s="21">
         <f>F53</f>
         <v>56629</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="27" t="s">
-        <v>196</v>
-      </c>
-      <c r="B63" s="36">
-        <f>IF(B62=0,"N/A",B61/B62)</f>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="B64" s="38">
+        <f>IF(B63=0,"N/A",B62/B63)</f>
         <v>-0.99</v>
       </c>
-      <c r="C63" s="36">
-        <f>IF(C62=0,"N/A",C61/C62)</f>
+      <c r="C64" s="38">
+        <f>IF(C63=0,"N/A",C62/C63)</f>
         <v>7.52</v>
       </c>
-      <c r="D63" s="36">
-        <f>IF(D62=0,"N/A",D61/D62)</f>
+      <c r="D64" s="38">
+        <f>IF(D63=0,"N/A",D62/D63)</f>
         <v>18.63</v>
       </c>
-      <c r="E63" s="36">
-        <f>IF(E62=0,"N/A",E61/E62)</f>
+      <c r="E64" s="38">
+        <f>IF(E63=0,"N/A",E62/E63)</f>
         <v>38.5</v>
       </c>
-      <c r="F63" s="36">
-        <f>IF(F62=0,"N/A",F61/F62)</f>
+      <c r="F64" s="38">
+        <f>IF(F63=0,"N/A",F62/F63)</f>
         <v>55.03</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="13" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B64" s="21" t="str">
+      <c r="B65" s="21" t="str">
         <f>Assumptions!B63</f>
         <v>0</v>
       </c>
-      <c r="C64" s="21">
-        <f>B65</f>
+      <c r="C65" s="21">
+        <f>B66</f>
         <v>-212164</v>
       </c>
-      <c r="D64" s="21">
-        <f>C65</f>
+      <c r="D65" s="21">
+        <f>C66</f>
         <v>222355</v>
       </c>
-      <c r="E64" s="21">
-        <f>D65</f>
+      <c r="E65" s="21">
+        <f>D66</f>
         <v>1485216</v>
       </c>
-      <c r="F64" s="21">
-        <f>E65</f>
+      <c r="F65" s="21">
+        <f>E66</f>
         <v>3608575</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="27" t="s">
-        <v>197</v>
-      </c>
-      <c r="B65" s="31">
-        <f>B64+B56</f>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="B66" s="31">
+        <f>B65+B56</f>
         <v>-212164</v>
       </c>
-      <c r="C65" s="31">
-        <f>C64+C56</f>
+      <c r="C66" s="31">
+        <f>C65+C56</f>
         <v>222355</v>
       </c>
-      <c r="D65" s="31">
-        <f>D64+D56</f>
+      <c r="D66" s="31">
+        <f>D65+D56</f>
         <v>1485216</v>
       </c>
-      <c r="E65" s="31">
-        <f>E64+E56</f>
+      <c r="E66" s="31">
+        <f>E65+E56</f>
         <v>3608575</v>
       </c>
-      <c r="F65" s="31">
-        <f>F64+F56</f>
+      <c r="F66" s="31">
+        <f>F65+F56</f>
         <v>6668055</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="B66" s="37">
-        <f>IF(B54=0,"",B65/B54*365)</f>
-        <v>-56</v>
-      </c>
-      <c r="C66" s="37">
-        <f>IF(C54=0,"",C65/C54*365)</f>
-        <v>46</v>
-      </c>
-      <c r="D66" s="37">
-        <f>IF(D54=0,"",D65/D54*365)</f>
-        <v>271</v>
-      </c>
-      <c r="E66" s="37">
-        <f>IF(E54=0,"",E65/E54*365)</f>
-        <v>593</v>
-      </c>
-      <c r="F66" s="37">
-        <f>IF(F54=0,"",F65/F54*365)</f>
-        <v>987</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="B67" s="38">
-        <f>IF(B54=0,"",B65/(B54/12))</f>
-        <v>-1.8</v>
-      </c>
-      <c r="C67" s="38">
-        <f>IF(C54=0,"",C65/(C54/12))</f>
-        <v>1.5</v>
-      </c>
-      <c r="D67" s="38">
-        <f>IF(D54=0,"",D65/(D54/12))</f>
-        <v>8.9</v>
-      </c>
-      <c r="E67" s="38">
-        <f>IF(E54=0,"",E65/(E54/12))</f>
-        <v>19.5</v>
-      </c>
-      <c r="F67" s="38">
-        <f>IF(F54=0,"",F65/(F54/12))</f>
-        <v>32.5</v>
+        <v>200</v>
+      </c>
+      <c r="B67" s="39">
+        <f>IF(B54=0,"",B66/B54*365)</f>
+        <v>-56</v>
+      </c>
+      <c r="C67" s="39">
+        <f>IF(C54=0,"",C66/C54*365)</f>
+        <v>46</v>
+      </c>
+      <c r="D67" s="39">
+        <f>IF(D54=0,"",D66/D54*365)</f>
+        <v>271</v>
+      </c>
+      <c r="E67" s="39">
+        <f>IF(E54=0,"",E66/E54*365)</f>
+        <v>593</v>
+      </c>
+      <c r="F67" s="39">
+        <f>IF(F54=0,"",F66/F54*365)</f>
+        <v>987</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="B68" s="35">
+        <v>201</v>
+      </c>
+      <c r="B68" s="40">
+        <f>IF(B54=0,"",B66/(B54/12))</f>
+        <v>-1.8</v>
+      </c>
+      <c r="C68" s="40">
+        <f>IF(C54=0,"",C66/(C54/12))</f>
+        <v>1.5</v>
+      </c>
+      <c r="D68" s="40">
+        <f>IF(D54=0,"",D66/(D54/12))</f>
+        <v>8.9</v>
+      </c>
+      <c r="E68" s="40">
+        <f>IF(E54=0,"",E66/(E54/12))</f>
+        <v>19.5</v>
+      </c>
+      <c r="F68" s="40">
+        <f>IF(F54=0,"",F66/(F54/12))</f>
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="B69" s="35">
         <f>IF(Assumptions!B12=0,"",B3/Assumptions!B12)</f>
         <v>0.2</v>
       </c>
-      <c r="C68" s="35">
+      <c r="C69" s="35">
         <f>IF(Assumptions!B12=0,"",C3/Assumptions!B12)</f>
         <v>0.33</v>
       </c>
-      <c r="D68" s="35">
+      <c r="D69" s="35">
         <f>IF(Assumptions!B12=0,"",D3/Assumptions!B12)</f>
         <v>0.5</v>
       </c>
-      <c r="E68" s="35">
+      <c r="E69" s="35">
         <f>IF(Assumptions!B12=0,"",E3/Assumptions!B12)</f>
         <v>0.67</v>
       </c>
-      <c r="F68" s="35">
+      <c r="F69" s="35">
         <f>IF(Assumptions!B12=0,"",F3/Assumptions!B12)</f>
         <v>0.83</v>
       </c>
     </row>
-    <row r="70" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="B70" s="12"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="12"/>
-      <c r="E70" s="12"/>
-      <c r="F70" s="12"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="B71" s="13" t="str">
-        <f>IF(B62=0,"N/A",IF(B63&gt;=1.2,"PASS","FAIL"))</f>
-        <v>FAIL</v>
-      </c>
-      <c r="C71" s="13" t="str">
-        <f>IF(C62=0,"N/A",IF(C63&gt;=1.2,"PASS","FAIL"))</f>
-        <v>PASS</v>
-      </c>
-      <c r="D71" s="13" t="str">
-        <f>IF(D62=0,"N/A",IF(D63&gt;=1.2,"PASS","FAIL"))</f>
-        <v>PASS</v>
-      </c>
-      <c r="E71" s="13" t="str">
-        <f>IF(E62=0,"N/A",IF(E63&gt;=1.2,"PASS","FAIL"))</f>
-        <v>PASS</v>
-      </c>
-      <c r="F71" s="13" t="str">
-        <f>IF(F62=0,"N/A",IF(F63&gt;=1.2,"PASS","FAIL"))</f>
-        <v>PASS</v>
-      </c>
+    <row r="71" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="B71" s="12"/>
+      <c r="C71" s="12"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="12"/>
+      <c r="F71" s="12"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B72" s="13" t="str">
+        <f>IF(B63=0,"N/A",IF(B64&gt;=1.2,"PASS","FAIL"))</f>
+        <v>FAIL</v>
+      </c>
+      <c r="C72" s="13" t="str">
+        <f>IF(C63=0,"N/A",IF(C64&gt;=1.2,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+      <c r="D72" s="13" t="str">
+        <f>IF(D63=0,"N/A",IF(D64&gt;=1.2,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+      <c r="E72" s="13" t="str">
+        <f>IF(E63=0,"N/A",IF(E64&gt;=1.2,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+      <c r="F72" s="13" t="str">
+        <f>IF(F63=0,"N/A",IF(F64&gt;=1.2,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B73" s="13" t="str">
         <f>IF(B56&gt;0,"PASS","FAIL")</f>
         <v>FAIL</v>
       </c>
-      <c r="C72" s="13" t="str">
+      <c r="C73" s="13" t="str">
         <f>IF(C56&gt;0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
-      <c r="D72" s="13" t="str">
+      <c r="D73" s="13" t="str">
         <f>IF(D56&gt;0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
-      <c r="E72" s="13" t="str">
+      <c r="E73" s="13" t="str">
         <f>IF(E56&gt;0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
-      <c r="F72" s="13" t="str">
+      <c r="F73" s="13" t="str">
         <f>IF(F56&gt;0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="B73" s="13" t="str">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="B74" s="13" t="str">
         <f>IF(Assumptions!B12=0,"N/A",IF(B3/Assumptions!B12&gt;=0.7,"PASS","FAIL"))</f>
         <v>FAIL</v>
       </c>
-      <c r="C73" s="13" t="str">
+      <c r="C74" s="13" t="str">
         <f>IF(Assumptions!B12=0,"N/A",IF(C3/Assumptions!B12&gt;=0.7,"PASS","FAIL"))</f>
         <v>FAIL</v>
       </c>
-      <c r="D73" s="13" t="str">
+      <c r="D74" s="13" t="str">
         <f>IF(Assumptions!B12=0,"N/A",IF(D3/Assumptions!B12&gt;=0.7,"PASS","FAIL"))</f>
         <v>FAIL</v>
       </c>
-      <c r="E73" s="13" t="str">
+      <c r="E74" s="13" t="str">
         <f>IF(Assumptions!B12=0,"N/A",IF(E3/Assumptions!B12&gt;=0.7,"PASS","FAIL"))</f>
         <v>FAIL</v>
       </c>
-      <c r="F73" s="13" t="str">
+      <c r="F74" s="13" t="str">
         <f>IF(Assumptions!B12=0,"N/A",IF(F3/Assumptions!B12&gt;=0.7,"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="B74" s="13" t="str">
-        <f>IF(B54=0,"N/A",IF(B65/(B54/12)&gt;=2,"PASS","FAIL"))</f>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="B75" s="13" t="str">
+        <f>IF(B54=0,"N/A",IF(B66/(B54/12)&gt;=2,"PASS","FAIL"))</f>
         <v>FAIL</v>
       </c>
-      <c r="C74" s="13" t="str">
-        <f>IF(C54=0,"N/A",IF(C65/(C54/12)&gt;=2,"PASS","FAIL"))</f>
+      <c r="C75" s="13" t="str">
+        <f>IF(C54=0,"N/A",IF(C66/(C54/12)&gt;=2,"PASS","FAIL"))</f>
         <v>FAIL</v>
       </c>
-      <c r="D74" s="13" t="str">
-        <f>IF(D54=0,"N/A",IF(D65/(D54/12)&gt;=2,"PASS","FAIL"))</f>
+      <c r="D75" s="13" t="str">
+        <f>IF(D54=0,"N/A",IF(D66/(D54/12)&gt;=2,"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
-      <c r="E74" s="13" t="str">
-        <f>IF(E54=0,"N/A",IF(E65/(E54/12)&gt;=2,"PASS","FAIL"))</f>
+      <c r="E75" s="13" t="str">
+        <f>IF(E54=0,"N/A",IF(E66/(E54/12)&gt;=2,"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
-      <c r="F74" s="13" t="str">
-        <f>IF(F54=0,"N/A",IF(F65/(F54/12)&gt;=2,"PASS","FAIL"))</f>
+      <c r="F75" s="13" t="str">
+        <f>IF(F54=0,"N/A",IF(F66/(F54/12)&gt;=2,"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
     </row>
-    <row r="76" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="12" t="s">
-        <v>206</v>
-      </c>
-      <c r="B76" s="12"/>
-      <c r="C76" s="12"/>
-      <c r="D76" s="12"/>
-      <c r="E76" s="12"/>
-      <c r="F76" s="12"/>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="B77" s="21">
+    <row r="77" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="B77" s="12"/>
+      <c r="C77" s="12"/>
+      <c r="D77" s="12"/>
+      <c r="E77" s="12"/>
+      <c r="F77" s="12"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B78" s="21">
         <f>IF(B3=0,"",B12/B3)</f>
         <v>9819</v>
       </c>
-      <c r="C77" s="21">
+      <c r="C78" s="21">
         <f>IF(C3=0,"",C12/C3)</f>
         <v>11063</v>
       </c>
-      <c r="D77" s="21">
+      <c r="D78" s="21">
         <f>IF(D3=0,"",D12/D3)</f>
         <v>10885</v>
       </c>
-      <c r="E77" s="21">
+      <c r="E78" s="21">
         <f>IF(E3=0,"",E12/E3)</f>
         <v>10857</v>
       </c>
-      <c r="F77" s="21">
+      <c r="F78" s="21">
         <f>IF(F3=0,"",F12/F3)</f>
         <v>11049</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="B78" s="21">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B79" s="21">
         <f>IF(B3=0,"",B54/B3)</f>
         <v>11587</v>
       </c>
-      <c r="C78" s="21">
+      <c r="C79" s="21">
         <f>IF(C3=0,"",C54/C3)</f>
         <v>8891</v>
       </c>
-      <c r="D78" s="21">
+      <c r="D79" s="21">
         <f>IF(D3=0,"",D54/D3)</f>
         <v>6676</v>
       </c>
-      <c r="E78" s="21">
+      <c r="E79" s="21">
         <f>IF(E3=0,"",E54/E3)</f>
         <v>5549</v>
       </c>
-      <c r="F78" s="21">
+      <c r="F79" s="21">
         <f>IF(F3=0,"",F54/F3)</f>
         <v>4930</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="B79" s="21">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="B80" s="21">
         <f>B51+B53</f>
         <v>887164</v>
       </c>
-      <c r="C79" s="21">
+      <c r="C80" s="21">
         <f>C51+C53</f>
         <v>1003271</v>
       </c>
-      <c r="D79" s="21">
+      <c r="D80" s="21">
         <f>D51+D53</f>
         <v>1008271</v>
       </c>
-      <c r="E79" s="21">
+      <c r="E80" s="21">
         <f>E51+E53</f>
         <v>993271</v>
       </c>
-      <c r="F79" s="21">
+      <c r="F80" s="21">
         <f>F51+F53</f>
         <v>993271</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="13" t="s">
-        <v>210</v>
-      </c>
-      <c r="B80" s="21">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="B81" s="21">
         <f>IF(B3=0,"",B52/B3)</f>
         <v>4194</v>
       </c>
-      <c r="C80" s="21">
+      <c r="C81" s="21">
         <f>IF(C3=0,"",C52/C3)</f>
         <v>3874</v>
       </c>
-      <c r="D80" s="21">
+      <c r="D81" s="21">
         <f>IF(D3=0,"",D52/D3)</f>
         <v>3315</v>
       </c>
-      <c r="E80" s="21">
+      <c r="E81" s="21">
         <f>IF(E3=0,"",E52/E3)</f>
         <v>3066</v>
       </c>
-      <c r="F80" s="21">
+      <c r="F81" s="21">
         <f>IF(F3=0,"",F52/F3)</f>
         <v>2944</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="B81" s="21">
-        <f>IF(B3=0,"",B77-B80)</f>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="B82" s="21">
+        <f>IF(B3=0,"",B78-B81)</f>
         <v>5625</v>
       </c>
-      <c r="C81" s="21">
-        <f>IF(C3=0,"",C77-C80)</f>
+      <c r="C82" s="21">
+        <f>IF(C3=0,"",C78-C81)</f>
         <v>7189</v>
       </c>
-      <c r="D81" s="21">
-        <f>IF(D3=0,"",D77-D80)</f>
+      <c r="D82" s="21">
+        <f>IF(D3=0,"",D78-D81)</f>
         <v>7570</v>
       </c>
-      <c r="E81" s="21">
-        <f>IF(E3=0,"",E77-E80)</f>
+      <c r="E82" s="21">
+        <f>IF(E3=0,"",E78-E81)</f>
         <v>7792</v>
       </c>
-      <c r="F81" s="21">
-        <f>IF(F3=0,"",F77-F80)</f>
+      <c r="F82" s="21">
+        <f>IF(F3=0,"",F78-F81)</f>
         <v>8106</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="39" t="s">
-        <v>212</v>
-      </c>
-      <c r="B82" s="40">
-        <f>IF(B81&lt;=0,"N/A",ROUNDUP(B79/B81,0))</f>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="41" t="s">
+        <v>214</v>
+      </c>
+      <c r="B83" s="42">
+        <f>IF(B82&lt;=0,"N/A",ROUNDUP(B80/B82,0))</f>
         <v>158</v>
       </c>
-      <c r="C82" s="40">
-        <f>IF(C81&lt;=0,"N/A",ROUNDUP(C79/C81,0))</f>
+      <c r="C83" s="42">
+        <f>IF(C82&lt;=0,"N/A",ROUNDUP(C80/C82,0))</f>
         <v>140</v>
       </c>
-      <c r="D82" s="40">
-        <f>IF(D81&lt;=0,"N/A",ROUNDUP(D79/D81,0))</f>
+      <c r="D83" s="42">
+        <f>IF(D82&lt;=0,"N/A",ROUNDUP(D80/D82,0))</f>
         <v>134</v>
       </c>
-      <c r="E82" s="40">
-        <f>IF(E81&lt;=0,"N/A",ROUNDUP(E79/E81,0))</f>
+      <c r="E83" s="42">
+        <f>IF(E82&lt;=0,"N/A",ROUNDUP(E80/E82,0))</f>
         <v>128</v>
       </c>
-      <c r="F82" s="40">
-        <f>IF(F81&lt;=0,"N/A",ROUNDUP(F79/F81,0))</f>
+      <c r="F83" s="42">
+        <f>IF(F82&lt;=0,"N/A",ROUNDUP(F80/F82,0))</f>
         <v>123</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" s="26" t="s">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="B84" s="26"/>
-      <c r="C84" s="26"/>
-      <c r="D84" s="26"/>
-      <c r="E84" s="26"/>
-      <c r="F84" s="26"/>
+      <c r="B85" s="26"/>
+      <c r="C85" s="26"/>
+      <c r="D85" s="26"/>
+      <c r="E85" s="26"/>
+      <c r="F85" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A85:F85"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
@@ -4654,7 +4683,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -4678,40 +4707,40 @@
         <v>46</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H2" s="25" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I2" s="25" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J2" s="25" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K2" s="25" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L2" s="25" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M2" s="25" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="N2" s="25" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -5497,7 +5526,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B24" s="21">
         <v>6500</v>
@@ -5605,7 +5634,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B27" s="21">
         <v>4500</v>
@@ -5713,7 +5742,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B30" s="21">
         <v>22000</v>
@@ -5758,7 +5787,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B31" s="21">
         <v>3000</v>
@@ -5803,7 +5832,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B32" s="21">
         <v>1833</v>
@@ -5911,7 +5940,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B35" s="21">
         <v>2500</v>
@@ -5956,7 +5985,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B36" s="21">
         <v>1000</v>
@@ -6001,7 +6030,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B37" s="21">
         <v>1500</v>
@@ -6046,7 +6075,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B38" s="21">
         <v>7500</v>
@@ -6198,7 +6227,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="27" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B42" s="21">
         <v>8886</v>
@@ -6248,7 +6277,7 @@
     </row>
     <row r="44" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B44" s="12"/>
       <c r="C44" s="12"/>
@@ -6323,7 +6352,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="27" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B46" s="31">
         <f>B10-B45</f>
@@ -6380,7 +6409,7 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="27" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B47" s="31">
         <f>0+B46</f>
@@ -6437,7 +6466,7 @@
     </row>
     <row r="49" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B49" s="12"/>
       <c r="C49" s="12"/>
@@ -6452,7 +6481,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B51" s="31">
         <f>M47</f>
@@ -6461,7 +6490,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B52" s="21">
         <f>MIN(B47:M47)</f>
@@ -6518,7 +6547,7 @@
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -6528,147 +6557,147 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="41" t="s">
-        <v>243</v>
-      </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
+      <c r="B3" s="43" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="42" t="s">
-        <v>244</v>
-      </c>
-      <c r="D4" s="43" t="s">
-        <v>245</v>
-      </c>
-      <c r="F4" s="44" t="s">
+      <c r="B4" s="44" t="s">
         <v>246</v>
+      </c>
+      <c r="D4" s="45" t="s">
+        <v>247</v>
+      </c>
+      <c r="F4" s="46" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="C7" s="45">
+        <v>256</v>
+      </c>
+      <c r="C7" s="47">
         <v>120</v>
       </c>
-      <c r="D7" s="45">
+      <c r="D7" s="47">
         <v>200</v>
       </c>
-      <c r="E7" s="45">
+      <c r="E7" s="47">
         <v>300</v>
       </c>
-      <c r="F7" s="45">
+      <c r="F7" s="47">
         <v>400</v>
       </c>
-      <c r="G7" s="45">
+      <c r="G7" s="47">
         <v>500</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="C8" s="46">
+        <v>257</v>
+      </c>
+      <c r="C8" s="48">
         <v>1414000</v>
       </c>
-      <c r="D8" s="46">
+      <c r="D8" s="48">
         <v>2212650</v>
       </c>
-      <c r="E8" s="46">
+      <c r="E8" s="48">
         <v>3265600</v>
       </c>
-      <c r="F8" s="46">
+      <c r="F8" s="48">
         <v>4342850</v>
       </c>
-      <c r="G8" s="46">
+      <c r="G8" s="48">
         <v>5524700</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="13" t="s">
-        <v>256</v>
-      </c>
-      <c r="C9" s="46">
+        <v>258</v>
+      </c>
+      <c r="C9" s="48">
         <v>780535</v>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="48">
         <v>936642</v>
       </c>
-      <c r="E9" s="46">
+      <c r="E9" s="48">
         <v>936642</v>
       </c>
-      <c r="F9" s="46">
+      <c r="F9" s="48">
         <v>936642</v>
       </c>
-      <c r="G9" s="46">
+      <c r="G9" s="48">
         <v>936642</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="C10" s="46">
+        <v>259</v>
+      </c>
+      <c r="C10" s="48">
         <v>604000</v>
       </c>
-      <c r="D10" s="46">
+      <c r="D10" s="48">
         <v>774860</v>
       </c>
-      <c r="E10" s="46">
+      <c r="E10" s="48">
         <v>994467.6</v>
       </c>
-      <c r="F10" s="46">
+      <c r="F10" s="48">
         <v>1226219.9279999998</v>
       </c>
-      <c r="G10" s="46">
+      <c r="G10" s="48">
         <v>1471949.32584</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="C11" s="46">
+        <v>197</v>
+      </c>
+      <c r="C11" s="48">
         <v>46628.6108154935</v>
       </c>
-      <c r="D11" s="46">
+      <c r="D11" s="48">
         <v>46628.6108154935</v>
       </c>
-      <c r="E11" s="46">
+      <c r="E11" s="48">
         <v>46628.6108154935</v>
       </c>
-      <c r="F11" s="46">
+      <c r="F11" s="48">
         <v>46628.6108154935</v>
       </c>
-      <c r="G11" s="46">
+      <c r="G11" s="48">
         <v>46628.6108154935</v>
       </c>
     </row>
@@ -6676,379 +6705,379 @@
       <c r="B12" s="27" t="s">
         <v>190</v>
       </c>
-      <c r="C12" s="47">
+      <c r="C12" s="49">
         <v>-17163.6108154935</v>
       </c>
-      <c r="D12" s="48">
+      <c r="D12" s="50">
         <v>454519.3891845065</v>
       </c>
-      <c r="E12" s="48">
+      <c r="E12" s="50">
         <v>1287861.7891845065</v>
       </c>
-      <c r="F12" s="48">
+      <c r="F12" s="50">
         <v>2133359.461184507</v>
       </c>
-      <c r="G12" s="48">
+      <c r="G12" s="50">
         <v>3069480.0633445065</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="27" t="s">
-        <v>197</v>
-      </c>
-      <c r="C13" s="47">
+        <v>199</v>
+      </c>
+      <c r="C13" s="49">
         <v>-17163.6108154935</v>
       </c>
-      <c r="D13" s="48">
+      <c r="D13" s="50">
         <v>437355.778369013</v>
       </c>
-      <c r="E13" s="48">
+      <c r="E13" s="50">
         <v>1725217.5675535195</v>
       </c>
-      <c r="F13" s="48">
+      <c r="F13" s="50">
         <v>3858577.0287380265</v>
       </c>
-      <c r="G13" s="48">
+      <c r="G13" s="50">
         <v>6928057.092082533</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="C14" s="49">
+        <v>260</v>
+      </c>
+      <c r="C14" s="51">
         <v>-0.0121383386248186</v>
       </c>
-      <c r="D14" s="50">
+      <c r="D14" s="52">
         <v>0.20541856560436875</v>
       </c>
-      <c r="E14" s="50">
+      <c r="E14" s="52">
         <v>0.39437217944160535</v>
       </c>
-      <c r="F14" s="50">
+      <c r="F14" s="52">
         <v>0.49123489440908774</v>
       </c>
-      <c r="G14" s="50">
+      <c r="G14" s="52">
         <v>0.555592170315946</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C15" s="51">
+        <v>261</v>
+      </c>
+      <c r="C15" s="53">
         <v>11783.333333333334</v>
       </c>
-      <c r="D15" s="51">
+      <c r="D15" s="53">
         <v>11063.25</v>
       </c>
-      <c r="E15" s="51">
+      <c r="E15" s="53">
         <v>10885.333333333334</v>
       </c>
-      <c r="F15" s="51">
+      <c r="F15" s="53">
         <v>10857.125</v>
       </c>
-      <c r="G15" s="51">
+      <c r="G15" s="53">
         <v>11049.4</v>
       </c>
-      <c r="H15" s="52" t="s">
-        <v>260</v>
+      <c r="H15" s="54" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="27" t="s">
-        <v>261</v>
-      </c>
-      <c r="C16" s="53">
+        <v>263</v>
+      </c>
+      <c r="C16" s="55">
         <v>0.5520049504950495</v>
       </c>
-      <c r="D16" s="50">
+      <c r="D16" s="52">
         <v>0.4233123178089621</v>
       </c>
-      <c r="E16" s="50">
+      <c r="E16" s="52">
         <v>0.2868207986281235</v>
       </c>
-      <c r="F16" s="50">
+      <c r="F16" s="52">
         <v>0.21567449946463726</v>
       </c>
-      <c r="G16" s="50">
+      <c r="G16" s="52">
         <v>0.16953716943906458</v>
       </c>
-      <c r="H16" s="52" t="s">
-        <v>262</v>
+      <c r="H16" s="54" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="C17" s="50">
+        <v>265</v>
+      </c>
+      <c r="C17" s="52">
         <v>0.12814710042432814</v>
       </c>
-      <c r="D17" s="50">
+      <c r="D17" s="52">
         <v>0.10505864009219713</v>
       </c>
-      <c r="E17" s="50">
+      <c r="E17" s="52">
         <v>0.09135848848603624</v>
       </c>
-      <c r="F17" s="50">
+      <c r="F17" s="52">
         <v>0.08470612118769931</v>
       </c>
-      <c r="G17" s="50">
+      <c r="G17" s="52">
         <v>0.07992919031838833</v>
       </c>
-      <c r="H17" s="52" t="s">
-        <v>264</v>
+      <c r="H17" s="54" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="27" t="s">
-        <v>265</v>
-      </c>
-      <c r="C18" s="53">
+        <v>267</v>
+      </c>
+      <c r="C18" s="55">
         <v>0.020838048090523337</v>
       </c>
-      <c r="D18" s="50">
+      <c r="D18" s="52">
         <v>0.22649221521704743</v>
       </c>
-      <c r="E18" s="50">
+      <c r="E18" s="52">
         <v>0.40865090641842233</v>
       </c>
-      <c r="F18" s="50">
+      <c r="F18" s="52">
         <v>0.5019717632430317</v>
       </c>
-      <c r="G18" s="50">
+      <c r="G18" s="52">
         <v>0.5640321961663076</v>
       </c>
-      <c r="H18" s="52" t="s">
-        <v>266</v>
+      <c r="H18" s="54" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="27" t="s">
-        <v>267</v>
-      </c>
-      <c r="C19" s="54">
-        <v>1</v>
-      </c>
-      <c r="D19" s="54"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="54"/>
-      <c r="H19" s="52" t="s">
-        <v>268</v>
+        <v>269</v>
+      </c>
+      <c r="C19" s="56">
+        <v>3</v>
+      </c>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="56"/>
+      <c r="G19" s="56"/>
+      <c r="H19" s="54" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="27" t="s">
-        <v>269</v>
-      </c>
-      <c r="C20" s="55">
+        <v>271</v>
+      </c>
+      <c r="C20" s="57">
         <v>0.6319081672107103</v>
       </c>
-      <c r="D20" s="56">
+      <c r="D20" s="58">
         <v>10.747650235238861</v>
       </c>
-      <c r="E20" s="56">
+      <c r="E20" s="58">
         <v>28.61956160951256</v>
       </c>
-      <c r="F20" s="56">
+      <c r="F20" s="58">
         <v>46.752155680255555</v>
       </c>
-      <c r="G20" s="56">
+      <c r="G20" s="58">
         <v>66.82825457722186</v>
       </c>
-      <c r="H20" s="52" t="s">
-        <v>270</v>
+      <c r="H20" s="54" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="27" t="s">
-        <v>271</v>
-      </c>
-      <c r="C21" s="57" t="s">
-        <v>249</v>
-      </c>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="52" t="s">
-        <v>248</v>
+        <v>273</v>
+      </c>
+      <c r="C21" s="59" t="s">
+        <v>251</v>
+      </c>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
+      <c r="H21" s="54" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="C22" s="58" t="s">
-        <v>273</v>
-      </c>
-      <c r="D22" s="58"/>
-      <c r="E22" s="58"/>
-      <c r="F22" s="58"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="52" t="s">
         <v>274</v>
+      </c>
+      <c r="C22" s="60" t="s">
+        <v>275</v>
+      </c>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="54" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="12" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E24" s="12"/>
       <c r="F24" s="12" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
     </row>
     <row r="25" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="59" t="s">
-        <v>279</v>
-      </c>
-      <c r="C25" s="60" t="s">
-        <v>280</v>
-      </c>
-      <c r="D25" s="61" t="s">
+      <c r="B25" s="61" t="s">
         <v>281</v>
       </c>
-      <c r="E25" s="61"/>
-      <c r="F25" s="62" t="s">
+      <c r="C25" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="G25" s="62"/>
-      <c r="H25" s="62"/>
+      <c r="D25" s="62" t="s">
+        <v>283</v>
+      </c>
+      <c r="E25" s="62"/>
+      <c r="F25" s="63" t="s">
+        <v>284</v>
+      </c>
+      <c r="G25" s="63"/>
+      <c r="H25" s="63"/>
     </row>
     <row r="26" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="59" t="s">
-        <v>283</v>
-      </c>
-      <c r="C26" s="63" t="s">
-        <v>284</v>
-      </c>
-      <c r="D26" s="61" t="s">
+      <c r="B26" s="61" t="s">
         <v>285</v>
       </c>
-      <c r="E26" s="61"/>
-      <c r="F26" s="62" t="s">
+      <c r="C26" s="64" t="s">
         <v>286</v>
       </c>
-      <c r="G26" s="62"/>
-      <c r="H26" s="62"/>
+      <c r="D26" s="62" t="s">
+        <v>287</v>
+      </c>
+      <c r="E26" s="62"/>
+      <c r="F26" s="63" t="s">
+        <v>288</v>
+      </c>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63"/>
     </row>
     <row r="27" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B27" s="59" t="s">
-        <v>287</v>
-      </c>
-      <c r="C27" s="60" t="s">
-        <v>280</v>
-      </c>
-      <c r="D27" s="61" t="s">
-        <v>288</v>
-      </c>
-      <c r="E27" s="61"/>
-      <c r="F27" s="62" t="s">
+      <c r="B27" s="61" t="s">
         <v>289</v>
       </c>
-      <c r="G27" s="62"/>
-      <c r="H27" s="62"/>
+      <c r="C27" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D27" s="62" t="s">
+        <v>290</v>
+      </c>
+      <c r="E27" s="62"/>
+      <c r="F27" s="63" t="s">
+        <v>291</v>
+      </c>
+      <c r="G27" s="63"/>
+      <c r="H27" s="63"/>
     </row>
     <row r="28" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="59" t="s">
-        <v>290</v>
-      </c>
-      <c r="C28" s="60" t="s">
-        <v>280</v>
-      </c>
-      <c r="D28" s="61" t="s">
-        <v>291</v>
-      </c>
-      <c r="E28" s="61"/>
-      <c r="F28" s="62" t="s">
+      <c r="B28" s="61" t="s">
         <v>292</v>
       </c>
-      <c r="G28" s="62"/>
-      <c r="H28" s="62"/>
+      <c r="C28" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D28" s="62" t="s">
+        <v>293</v>
+      </c>
+      <c r="E28" s="62"/>
+      <c r="F28" s="63" t="s">
+        <v>294</v>
+      </c>
+      <c r="G28" s="63"/>
+      <c r="H28" s="63"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="59" t="s">
-        <v>293</v>
-      </c>
-      <c r="C29" s="60" t="s">
-        <v>280</v>
-      </c>
-      <c r="D29" s="61" t="s">
-        <v>294</v>
-      </c>
-      <c r="E29" s="61"/>
-      <c r="F29" s="62" t="s">
+      <c r="B29" s="61" t="s">
         <v>295</v>
       </c>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
+      <c r="C29" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D29" s="62" t="s">
+        <v>296</v>
+      </c>
+      <c r="E29" s="62"/>
+      <c r="F29" s="63" t="s">
+        <v>297</v>
+      </c>
+      <c r="G29" s="63"/>
+      <c r="H29" s="63"/>
     </row>
     <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="59" t="s">
-        <v>296</v>
-      </c>
-      <c r="C30" s="60" t="s">
-        <v>280</v>
-      </c>
-      <c r="D30" s="61" t="s">
-        <v>297</v>
-      </c>
-      <c r="E30" s="61"/>
-      <c r="F30" s="62" t="s">
+      <c r="B30" s="61" t="s">
         <v>298</v>
       </c>
-      <c r="G30" s="62"/>
-      <c r="H30" s="62"/>
+      <c r="C30" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D30" s="62" t="s">
+        <v>299</v>
+      </c>
+      <c r="E30" s="62"/>
+      <c r="F30" s="63" t="s">
+        <v>300</v>
+      </c>
+      <c r="G30" s="63"/>
+      <c r="H30" s="63"/>
     </row>
     <row r="31" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B31" s="59" t="s">
-        <v>299</v>
-      </c>
-      <c r="C31" s="60" t="s">
-        <v>280</v>
-      </c>
-      <c r="D31" s="61" t="s">
-        <v>300</v>
-      </c>
-      <c r="E31" s="61"/>
-      <c r="F31" s="62" t="s">
+      <c r="B31" s="61" t="s">
         <v>301</v>
       </c>
-      <c r="G31" s="62"/>
-      <c r="H31" s="62"/>
+      <c r="C31" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D31" s="62" t="s">
+        <v>302</v>
+      </c>
+      <c r="E31" s="62"/>
+      <c r="F31" s="63" t="s">
+        <v>303</v>
+      </c>
+      <c r="G31" s="63"/>
+      <c r="H31" s="63"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="59" t="s">
-        <v>302</v>
+      <c r="B33" s="61" t="s">
+        <v>304</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D33" s="27"/>
       <c r="E33" s="27"/>
       <c r="F33" s="27"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="64" t="s">
+      <c r="B35" s="65" t="s">
         <v>155</v>
       </c>
-      <c r="C35" s="64"/>
-      <c r="D35" s="64"/>
-      <c r="E35" s="64"/>
-      <c r="F35" s="64"/>
-      <c r="G35" s="64"/>
-      <c r="H35" s="64"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="23">

</xml_diff>

<commit_message>
Wire cumNIRef to all 5 addDashboardSheet call sites for formula-linked break-even
- underwriting-workbook.ts: destructure cumNIRow from buildOperatingStatement,
  pass cumNIRef with sheetName "5-Year Operating Stmt"
- formula-export.ts: add cumNIRow to FiveYearResult interface and return value,
  pass fiveYr.cumNIRow as cumNIRef with sheetName "5-Year Model"
- excel-export.ts: pass cumNIRef with sheetName "Financial Model", row 8
- lender-proforma-export.ts: pass cumNIRef with sheetName "5-Year P&L", row 19
- underwriting-export.ts: return cumNIRow from buildFiveYearPL, wire both
  call sites with sheetName "5-Year P&L"

All QA suites pass: 24/24 excel, 33/33 parity.
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="306">
   <si>
     <t>How to Use This Workbook</t>
   </si>
@@ -1250,7 +1250,9 @@
     <xf numFmtId="167" fontId="12" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6895,13 +6897,26 @@
       <c r="B21" s="27" t="s">
         <v>273</v>
       </c>
-      <c r="C21" s="59" t="s">
-        <v>251</v>
-      </c>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="59"/>
+      <c r="C21" s="59" t="str">
+        <f>IF('5-Year Model'!B58&gt;=0,"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="37" t="str">
+        <f>IF('5-Year Model'!C58&gt;=0,"✓ Break-even","")</f>
+        <v>✓ Break-even</v>
+      </c>
+      <c r="E21" s="59" t="str">
+        <f>IF('5-Year Model'!D58&gt;=0,"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="59" t="str">
+        <f>IF('5-Year Model'!E58&gt;=0,"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="59" t="str">
+        <f>IF('5-Year Model'!F58&gt;=0,"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
       <c r="H21" s="54" t="s">
         <v>250</v>
       </c>
@@ -7080,11 +7095,10 @@
       <c r="H35" s="65"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="22">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C21:G21"/>
     <mergeCell ref="C22:G22"/>
     <mergeCell ref="D24:E24"/>
     <mergeCell ref="F24:H24"/>
@@ -7165,10 +7179,10 @@
       <formula>C17&lt;=0.15</formula>
     </cfRule>
     <cfRule type="expression" dxfId="16" priority="2">
-      <formula>C17&lt;=0.25</formula>
+      <formula>C17&lt;=0.22</formula>
     </cfRule>
     <cfRule type="expression" dxfId="17" priority="3">
-      <formula>C17&gt;0.25</formula>
+      <formula>C17&gt;0.22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18:G18">

</xml_diff>

<commit_message>
Merged changes from m1t3inxu/main
Replit-Task-Id: f8b3c7d7-0638-4d08-8913-c99186c994b9
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'5-Year Model'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Year 1 Pro Forma'!$A1:$N54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Year 1 Pro Forma'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Financial Health'!$A1:$H40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Financial Health'!$A1:$H35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Financial Health'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="305">
   <si>
     <t>How to Use This Workbook</t>
   </si>
@@ -818,21 +818,6 @@
     <t>≥ $10,000</t>
   </si>
   <si>
-    <t>Cost per Student</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Instructional / Student</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Facility / Student</t>
-  </si>
-  <si>
-    <t>≤ $2,000 / $2k–$3.5k / &gt; $3,500</t>
-  </si>
-  <si>
-    <t>Surplus per Student</t>
-  </si>
-  <si>
     <t>Payroll %</t>
   </si>
   <si>
@@ -870,9 +855,6 @@
   </si>
   <si>
     <t>≥ 24 months</t>
-  </si>
-  <si>
-    <t>≥ 90 days</t>
   </si>
   <si>
     <t>FINANCIAL HEALTH SIGNALS</t>
@@ -1173,7 +1155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1255,18 +1237,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="166" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -6571,7 +6541,7 @@
     <tabColor rgb="FF328555"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H40"/>
+  <dimension ref="B2:H35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -6820,458 +6790,352 @@
         <v>262</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="27" t="s">
         <v>263</v>
       </c>
       <c r="C16" s="55">
-        <v>11926.363423462444</v>
-      </c>
-      <c r="D16" s="55">
-        <v>8790.653054077467</v>
-      </c>
-      <c r="E16" s="55">
-        <v>6592.460702718312</v>
-      </c>
-      <c r="F16" s="55">
-        <v>5523.726347038733</v>
-      </c>
-      <c r="G16" s="55">
-        <v>4910.4398733109865</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="13" t="s">
+        <v>0.5520049504950495</v>
+      </c>
+      <c r="D16" s="52">
+        <v>0.4233123178089621</v>
+      </c>
+      <c r="E16" s="52">
+        <v>0.2868207986281235</v>
+      </c>
+      <c r="F16" s="52">
+        <v>0.21567449946463726</v>
+      </c>
+      <c r="G16" s="52">
+        <v>0.16953716943906458</v>
+      </c>
+      <c r="H16" s="54" t="s">
         <v>264</v>
       </c>
-      <c r="C17" s="48">
-        <v>650</v>
-      </c>
-      <c r="D17" s="48">
-        <v>670</v>
-      </c>
-      <c r="E17" s="48">
-        <v>690</v>
-      </c>
-      <c r="F17" s="48">
-        <v>710</v>
-      </c>
-      <c r="G17" s="48">
-        <v>732</v>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="C17" s="51">
+        <v>0.22772277227722773</v>
+      </c>
+      <c r="D17" s="52">
+        <v>0.1498926626443405</v>
+      </c>
+      <c r="E17" s="52">
+        <v>0.10460975012248896</v>
+      </c>
+      <c r="F17" s="52">
+        <v>0.08101959036116835</v>
+      </c>
+      <c r="G17" s="52">
+        <v>0.06559982005176752</v>
+      </c>
+      <c r="H17" s="54" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="C18" s="56">
-        <v>2683.3333333333335</v>
-      </c>
-      <c r="D18" s="53">
-        <v>1658.3</v>
-      </c>
-      <c r="E18" s="53">
-        <v>1138.712</v>
-      </c>
-      <c r="F18" s="53">
-        <v>879.6398199999999</v>
-      </c>
-      <c r="G18" s="53">
-        <v>724.8386516800001</v>
+      <c r="B18" s="27" t="s">
+        <v>267</v>
+      </c>
+      <c r="C18" s="55">
+        <v>0.020838048090523337</v>
+      </c>
+      <c r="D18" s="52">
+        <v>0.22649221521704743</v>
+      </c>
+      <c r="E18" s="52">
+        <v>0.40865090641842233</v>
+      </c>
+      <c r="F18" s="52">
+        <v>0.5019717632430317</v>
+      </c>
+      <c r="G18" s="52">
+        <v>0.5640321961663076</v>
       </c>
       <c r="H18" s="54" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="27" t="s">
-        <v>267</v>
-      </c>
-      <c r="C19" s="57">
-        <v>-143.0300901291125</v>
-      </c>
-      <c r="D19" s="58">
-        <v>2272.5969459225325</v>
-      </c>
-      <c r="E19" s="58">
-        <v>4292.872630615022</v>
-      </c>
-      <c r="F19" s="58">
-        <v>5333.398652961267</v>
-      </c>
-      <c r="G19" s="58">
-        <v>6138.960126689013</v>
+        <v>269</v>
+      </c>
+      <c r="C19" s="56">
+        <v>3</v>
+      </c>
+      <c r="D19" s="56">
+        <v>3</v>
+      </c>
+      <c r="E19" s="56">
+        <v>3</v>
+      </c>
+      <c r="F19" s="56">
+        <v>3</v>
+      </c>
+      <c r="G19" s="56">
+        <v>3</v>
+      </c>
+      <c r="H19" s="54" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="27" t="s">
-        <v>268</v>
-      </c>
-      <c r="C20" s="59">
-        <v>0.5520049504950495</v>
-      </c>
-      <c r="D20" s="52">
-        <v>0.4233123178089621</v>
-      </c>
-      <c r="E20" s="52">
-        <v>0.2868207986281235</v>
-      </c>
-      <c r="F20" s="52">
-        <v>0.21567449946463726</v>
-      </c>
-      <c r="G20" s="52">
-        <v>0.16953716943906458</v>
+        <v>271</v>
+      </c>
+      <c r="C20" s="57">
+        <v>0.6319081672107103</v>
+      </c>
+      <c r="D20" s="58">
+        <v>10.747650235238861</v>
+      </c>
+      <c r="E20" s="58">
+        <v>28.61956160951256</v>
+      </c>
+      <c r="F20" s="58">
+        <v>46.752155680255555</v>
+      </c>
+      <c r="G20" s="58">
+        <v>66.82825457722186</v>
       </c>
       <c r="H20" s="54" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="27" t="s">
-        <v>270</v>
-      </c>
-      <c r="C21" s="51">
-        <v>0.22772277227722773</v>
-      </c>
-      <c r="D21" s="52">
-        <v>0.1498926626443405</v>
-      </c>
-      <c r="E21" s="52">
-        <v>0.10460975012248896</v>
-      </c>
-      <c r="F21" s="52">
-        <v>0.08101959036116835</v>
-      </c>
-      <c r="G21" s="52">
-        <v>0.06559982005176752</v>
+        <v>273</v>
+      </c>
+      <c r="C21" s="59" t="str">
+        <f>IF('5-Year Model'!B58&gt;=0,"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="37" t="str">
+        <f>IF(AND('5-Year Model'!C58&gt;=0,'5-Year Model'!B58&lt;0),"✓ Break-even","")</f>
+        <v>✓ Break-even</v>
+      </c>
+      <c r="E21" s="59" t="str">
+        <f>IF(AND('5-Year Model'!D58&gt;=0,'5-Year Model'!C58&lt;0),"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="59" t="str">
+        <f>IF(AND('5-Year Model'!E58&gt;=0,'5-Year Model'!D58&lt;0),"✓ Break-even","")</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="59" t="str">
+        <f>IF(AND('5-Year Model'!F58&gt;=0,'5-Year Model'!E58&lt;0),"✓ Break-even","")</f>
+        <v>0</v>
       </c>
       <c r="H21" s="54" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="C22" s="59">
-        <v>0.020838048090523337</v>
-      </c>
-      <c r="D22" s="52">
-        <v>0.22649221521704743</v>
-      </c>
-      <c r="E22" s="52">
-        <v>0.40865090641842233</v>
-      </c>
-      <c r="F22" s="52">
-        <v>0.5019717632430317</v>
-      </c>
-      <c r="G22" s="52">
-        <v>0.5640321961663076</v>
+        <v>274</v>
+      </c>
+      <c r="C22" s="60">
+        <v>0</v>
+      </c>
+      <c r="D22" s="60">
+        <v>3</v>
+      </c>
+      <c r="E22" s="60">
+        <v>10</v>
+      </c>
+      <c r="F22" s="61">
+        <v>21</v>
+      </c>
+      <c r="G22" s="56">
+        <v>34</v>
       </c>
       <c r="H22" s="54" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="27" t="s">
-        <v>274</v>
-      </c>
-      <c r="C23" s="60">
-        <v>3</v>
-      </c>
-      <c r="D23" s="60">
-        <v>3</v>
-      </c>
-      <c r="E23" s="60">
-        <v>3</v>
-      </c>
-      <c r="F23" s="60">
-        <v>3</v>
-      </c>
-      <c r="G23" s="60">
-        <v>3</v>
-      </c>
-      <c r="H23" s="54" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="27" t="s">
+    <row r="24" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="C24" s="61">
-        <v>0.6319081672107103</v>
-      </c>
-      <c r="D24" s="62">
-        <v>10.747650235238861</v>
-      </c>
-      <c r="E24" s="62">
-        <v>28.61956160951256</v>
-      </c>
-      <c r="F24" s="62">
-        <v>46.752155680255555</v>
-      </c>
-      <c r="G24" s="62">
-        <v>66.82825457722186</v>
-      </c>
-      <c r="H24" s="54" t="s">
+      <c r="C24" s="12" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="27" t="s">
+      <c r="D24" s="12" t="s">
         <v>278</v>
       </c>
-      <c r="C25" s="63" t="str">
-        <f>IF('5-Year Model'!B58&gt;=0,"✓ Break-even","")</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="37" t="str">
-        <f>IF(AND('5-Year Model'!C58&gt;=0,'5-Year Model'!B58&lt;0),"✓ Break-even","")</f>
-        <v>✓ Break-even</v>
-      </c>
-      <c r="E25" s="63" t="str">
-        <f>IF(AND('5-Year Model'!D58&gt;=0,'5-Year Model'!C58&lt;0),"✓ Break-even","")</f>
-        <v>0</v>
-      </c>
-      <c r="F25" s="63" t="str">
-        <f>IF(AND('5-Year Model'!E58&gt;=0,'5-Year Model'!D58&lt;0),"✓ Break-even","")</f>
-        <v>0</v>
-      </c>
-      <c r="G25" s="63" t="str">
-        <f>IF(AND('5-Year Model'!F58&gt;=0,'5-Year Model'!E58&lt;0),"✓ Break-even","")</f>
-        <v>0</v>
-      </c>
-      <c r="H25" s="54" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="27" t="s">
+      <c r="E24" s="12"/>
+      <c r="F24" s="12" t="s">
         <v>279</v>
       </c>
-      <c r="C26" s="64">
-        <v>0</v>
-      </c>
-      <c r="D26" s="64">
-        <v>3</v>
-      </c>
-      <c r="E26" s="64">
-        <v>10</v>
-      </c>
-      <c r="F26" s="65">
-        <v>21</v>
-      </c>
-      <c r="G26" s="60">
-        <v>34</v>
-      </c>
-      <c r="H26" s="54" t="s">
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="62" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B27" s="27" t="s">
-        <v>200</v>
-      </c>
-      <c r="C27" s="64">
-        <v>0</v>
-      </c>
-      <c r="D27" s="60">
-        <v>91</v>
-      </c>
-      <c r="E27" s="60">
-        <v>318</v>
-      </c>
-      <c r="F27" s="60">
-        <v>637</v>
-      </c>
-      <c r="G27" s="60">
-        <v>1030</v>
-      </c>
-      <c r="H27" s="54" t="s">
+      <c r="C25" s="37" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="12" t="s">
+      <c r="D25" s="63" t="s">
         <v>282</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="E25" s="63"/>
+      <c r="F25" s="64" t="s">
         <v>283</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="G25" s="64"/>
+      <c r="H25" s="64"/>
+    </row>
+    <row r="26" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="62" t="s">
         <v>284</v>
       </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12" t="s">
+      <c r="C26" s="65" t="s">
         <v>285</v>
       </c>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
+      <c r="D26" s="63" t="s">
+        <v>286</v>
+      </c>
+      <c r="E26" s="63"/>
+      <c r="F26" s="64" t="s">
+        <v>287</v>
+      </c>
+      <c r="G26" s="64"/>
+      <c r="H26" s="64"/>
+    </row>
+    <row r="27" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="62" t="s">
+        <v>288</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D27" s="63" t="s">
+        <v>289</v>
+      </c>
+      <c r="E27" s="63"/>
+      <c r="F27" s="64" t="s">
+        <v>290</v>
+      </c>
+      <c r="G27" s="64"/>
+      <c r="H27" s="64"/>
+    </row>
+    <row r="28" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="62" t="s">
+        <v>291</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D28" s="63" t="s">
+        <v>292</v>
+      </c>
+      <c r="E28" s="63"/>
+      <c r="F28" s="64" t="s">
+        <v>293</v>
+      </c>
+      <c r="G28" s="64"/>
+      <c r="H28" s="64"/>
+    </row>
+    <row r="29" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="62" t="s">
+        <v>294</v>
+      </c>
+      <c r="C29" s="37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D29" s="63" t="s">
+        <v>295</v>
+      </c>
+      <c r="E29" s="63"/>
+      <c r="F29" s="64" t="s">
+        <v>296</v>
+      </c>
+      <c r="G29" s="64"/>
+      <c r="H29" s="64"/>
     </row>
     <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="66" t="s">
-        <v>286</v>
+      <c r="B30" s="62" t="s">
+        <v>297</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D30" s="67" t="s">
-        <v>288</v>
-      </c>
-      <c r="E30" s="67"/>
-      <c r="F30" s="68" t="s">
-        <v>289</v>
-      </c>
-      <c r="G30" s="68"/>
-      <c r="H30" s="68"/>
+        <v>281</v>
+      </c>
+      <c r="D30" s="63" t="s">
+        <v>298</v>
+      </c>
+      <c r="E30" s="63"/>
+      <c r="F30" s="64" t="s">
+        <v>299</v>
+      </c>
+      <c r="G30" s="64"/>
+      <c r="H30" s="64"/>
     </row>
     <row r="31" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B31" s="66" t="s">
-        <v>290</v>
-      </c>
-      <c r="C31" s="69" t="s">
-        <v>291</v>
-      </c>
-      <c r="D31" s="67" t="s">
-        <v>292</v>
-      </c>
-      <c r="E31" s="67"/>
-      <c r="F31" s="68" t="s">
-        <v>293</v>
-      </c>
-      <c r="G31" s="68"/>
-      <c r="H31" s="68"/>
-    </row>
-    <row r="32" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B32" s="66" t="s">
-        <v>294</v>
-      </c>
-      <c r="C32" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D32" s="67" t="s">
-        <v>295</v>
-      </c>
-      <c r="E32" s="67"/>
-      <c r="F32" s="68" t="s">
-        <v>296</v>
-      </c>
-      <c r="G32" s="68"/>
-      <c r="H32" s="68"/>
-    </row>
-    <row r="33" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="66" t="s">
-        <v>297</v>
-      </c>
-      <c r="C33" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D33" s="67" t="s">
-        <v>298</v>
-      </c>
-      <c r="E33" s="67"/>
-      <c r="F33" s="68" t="s">
-        <v>299</v>
-      </c>
-      <c r="G33" s="68"/>
-      <c r="H33" s="68"/>
-    </row>
-    <row r="34" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="66" t="s">
+      <c r="B31" s="62" t="s">
         <v>300</v>
       </c>
-      <c r="C34" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D34" s="67" t="s">
+      <c r="C31" s="37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D31" s="63" t="s">
         <v>301</v>
       </c>
-      <c r="E34" s="67"/>
-      <c r="F34" s="68" t="s">
+      <c r="E31" s="63"/>
+      <c r="F31" s="64" t="s">
         <v>302</v>
       </c>
-      <c r="G34" s="68"/>
-      <c r="H34" s="68"/>
-    </row>
-    <row r="35" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G31" s="64"/>
+      <c r="H31" s="64"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="62" t="s">
+        <v>303</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="66" t="s">
-        <v>303</v>
-      </c>
-      <c r="C35" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D35" s="67" t="s">
-        <v>304</v>
-      </c>
-      <c r="E35" s="67"/>
-      <c r="F35" s="68" t="s">
-        <v>305</v>
-      </c>
-      <c r="G35" s="68"/>
-      <c r="H35" s="68"/>
-    </row>
-    <row r="36" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="66" t="s">
-        <v>306</v>
-      </c>
-      <c r="C36" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D36" s="67" t="s">
-        <v>307</v>
-      </c>
-      <c r="E36" s="67"/>
-      <c r="F36" s="68" t="s">
-        <v>308</v>
-      </c>
-      <c r="G36" s="68"/>
-      <c r="H36" s="68"/>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="66" t="s">
-        <v>309</v>
-      </c>
-      <c r="C38" s="27" t="s">
-        <v>310</v>
-      </c>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="70" t="s">
         <v>155</v>
       </c>
-      <c r="C40" s="70"/>
-      <c r="D40" s="70"/>
-      <c r="E40" s="70"/>
-      <c r="F40" s="70"/>
-      <c r="G40" s="70"/>
-      <c r="H40" s="70"/>
+      <c r="C35" s="66"/>
+      <c r="D35" s="66"/>
+      <c r="E35" s="66"/>
+      <c r="F35" s="66"/>
+      <c r="G35" s="66"/>
+      <c r="H35" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="20">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:H28"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="F29:H29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="F30:H30"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:H31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="B35:H35"/>
   </mergeCells>
   <conditionalFormatting sqref="C12:G12">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -7317,48 +7181,48 @@
       <formula>C15&lt;7000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C20:G20">
+  <conditionalFormatting sqref="C16:G16">
     <cfRule type="expression" dxfId="12" priority="1">
-      <formula>C20&lt;=0.55</formula>
+      <formula>C16&lt;=0.55</formula>
     </cfRule>
     <cfRule type="expression" dxfId="13" priority="2">
-      <formula>C20&lt;=0.65</formula>
+      <formula>C16&lt;=0.65</formula>
     </cfRule>
     <cfRule type="expression" dxfId="14" priority="3">
-      <formula>C20&gt;0.65</formula>
+      <formula>C16&gt;0.65</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21:G21">
+  <conditionalFormatting sqref="C17:G17">
     <cfRule type="expression" dxfId="15" priority="1">
-      <formula>C21&lt;=0.15</formula>
+      <formula>C17&lt;=0.15</formula>
     </cfRule>
     <cfRule type="expression" dxfId="16" priority="2">
-      <formula>C21&lt;=0.22</formula>
+      <formula>C17&lt;=0.22</formula>
     </cfRule>
     <cfRule type="expression" dxfId="17" priority="3">
-      <formula>C21&gt;0.22</formula>
+      <formula>C17&gt;0.22</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C22:G22">
+  <conditionalFormatting sqref="C18:G18">
     <cfRule type="expression" dxfId="18" priority="1">
-      <formula>C22&gt;=0.10</formula>
+      <formula>C18&gt;=0.10</formula>
     </cfRule>
     <cfRule type="expression" dxfId="19" priority="2">
-      <formula>C22&gt;=0</formula>
+      <formula>C18&gt;=0</formula>
     </cfRule>
     <cfRule type="expression" dxfId="20" priority="3">
-      <formula>C22&lt;0</formula>
+      <formula>C18&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24:G24">
+  <conditionalFormatting sqref="C20:G20">
     <cfRule type="expression" dxfId="21" priority="1">
-      <formula>C24&gt;=1.25</formula>
+      <formula>C20&gt;=1.25</formula>
     </cfRule>
     <cfRule type="expression" dxfId="22" priority="2">
-      <formula>C24&gt;=1</formula>
+      <formula>C20&gt;=1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="23" priority="3">
-      <formula>C24&lt;1</formula>
+      <formula>C20&lt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix corrupted Excel and PDF exports by handling binary data correctly
Refactored binary export routes in `models.ts` to use a new `sendBinary` helper function, ensuring correct `Content-Type`, `Content-Disposition`, and `Content-Length` headers are set, and utilizing `res.end()` to prevent Netlify proxy from re-encoding data as UTF-8. Also removed a duplicate and outdated API proxy rule from `_redirects`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b2544c49-db65-4b24-b7e9-889dfec662fa
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/NnIlujE
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'5-Year Model'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Year 1 Pro Forma'!$A1:$N54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Year 1 Pro Forma'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Financial Health'!$A1:$H35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Financial Health'!$A1:$H40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Financial Health'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="311">
   <si>
     <t>How to Use This Workbook</t>
   </si>
@@ -818,6 +818,21 @@
     <t>≥ $10,000</t>
   </si>
   <si>
+    <t>Cost per Student</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Instructional / Student</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Facility / Student</t>
+  </si>
+  <si>
+    <t>≤ $2,000 / $2k–$3.5k / &gt; $3,500</t>
+  </si>
+  <si>
+    <t>Surplus per Student</t>
+  </si>
+  <si>
     <t>Payroll %</t>
   </si>
   <si>
@@ -855,6 +870,9 @@
   </si>
   <si>
     <t>≥ 24 months</t>
+  </si>
+  <si>
+    <t>≥ 90 days</t>
   </si>
   <si>
     <t>FINANCIAL HEALTH SIGNALS</t>
@@ -1155,7 +1173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1237,6 +1255,18 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="166" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -6541,7 +6571,7 @@
     <tabColor rgb="FF328555"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H35"/>
+  <dimension ref="B2:H40"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -6790,352 +6820,458 @@
         <v>262</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="27" t="s">
         <v>263</v>
       </c>
       <c r="C16" s="55">
-        <v>0.5520049504950495</v>
-      </c>
-      <c r="D16" s="52">
-        <v>0.4233123178089621</v>
-      </c>
-      <c r="E16" s="52">
-        <v>0.2868207986281235</v>
-      </c>
-      <c r="F16" s="52">
-        <v>0.21567449946463726</v>
-      </c>
-      <c r="G16" s="52">
-        <v>0.16953716943906458</v>
-      </c>
-      <c r="H16" s="54" t="s">
+        <v>11926.363423462444</v>
+      </c>
+      <c r="D16" s="55">
+        <v>8790.653054077467</v>
+      </c>
+      <c r="E16" s="55">
+        <v>6592.460702718312</v>
+      </c>
+      <c r="F16" s="55">
+        <v>5523.726347038733</v>
+      </c>
+      <c r="G16" s="55">
+        <v>4910.4398733109865</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="13" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="27" t="s">
+      <c r="C17" s="48">
+        <v>650</v>
+      </c>
+      <c r="D17" s="48">
+        <v>670</v>
+      </c>
+      <c r="E17" s="48">
+        <v>690</v>
+      </c>
+      <c r="F17" s="48">
+        <v>710</v>
+      </c>
+      <c r="G17" s="48">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="C17" s="51">
-        <v>0.22772277227722773</v>
-      </c>
-      <c r="D17" s="52">
-        <v>0.1498926626443405</v>
-      </c>
-      <c r="E17" s="52">
-        <v>0.10460975012248896</v>
-      </c>
-      <c r="F17" s="52">
-        <v>0.08101959036116835</v>
-      </c>
-      <c r="G17" s="52">
-        <v>0.06559982005176752</v>
-      </c>
-      <c r="H17" s="54" t="s">
+      <c r="C18" s="56">
+        <v>2683.3333333333335</v>
+      </c>
+      <c r="D18" s="53">
+        <v>1658.3</v>
+      </c>
+      <c r="E18" s="53">
+        <v>1138.712</v>
+      </c>
+      <c r="F18" s="53">
+        <v>879.6398199999999</v>
+      </c>
+      <c r="G18" s="53">
+        <v>724.8386516800001</v>
+      </c>
+      <c r="H18" s="54" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="27" t="s">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="C18" s="55">
-        <v>0.020838048090523337</v>
-      </c>
-      <c r="D18" s="52">
-        <v>0.22649221521704743</v>
-      </c>
-      <c r="E18" s="52">
-        <v>0.40865090641842233</v>
-      </c>
-      <c r="F18" s="52">
-        <v>0.5019717632430317</v>
-      </c>
-      <c r="G18" s="52">
-        <v>0.5640321961663076</v>
-      </c>
-      <c r="H18" s="54" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="27" t="s">
-        <v>269</v>
-      </c>
-      <c r="C19" s="56">
-        <v>3</v>
-      </c>
-      <c r="D19" s="56">
-        <v>3</v>
-      </c>
-      <c r="E19" s="56">
-        <v>3</v>
-      </c>
-      <c r="F19" s="56">
-        <v>3</v>
-      </c>
-      <c r="G19" s="56">
-        <v>3</v>
-      </c>
-      <c r="H19" s="54" t="s">
-        <v>270</v>
+      <c r="C19" s="57">
+        <v>-143.0300901291125</v>
+      </c>
+      <c r="D19" s="58">
+        <v>2272.5969459225325</v>
+      </c>
+      <c r="E19" s="58">
+        <v>4292.872630615022</v>
+      </c>
+      <c r="F19" s="58">
+        <v>5333.398652961267</v>
+      </c>
+      <c r="G19" s="58">
+        <v>6138.960126689013</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="27" t="s">
-        <v>271</v>
-      </c>
-      <c r="C20" s="57">
-        <v>0.6319081672107103</v>
-      </c>
-      <c r="D20" s="58">
-        <v>10.747650235238861</v>
-      </c>
-      <c r="E20" s="58">
-        <v>28.61956160951256</v>
-      </c>
-      <c r="F20" s="58">
-        <v>46.752155680255555</v>
-      </c>
-      <c r="G20" s="58">
-        <v>66.82825457722186</v>
+        <v>268</v>
+      </c>
+      <c r="C20" s="59">
+        <v>0.5520049504950495</v>
+      </c>
+      <c r="D20" s="52">
+        <v>0.4233123178089621</v>
+      </c>
+      <c r="E20" s="52">
+        <v>0.2868207986281235</v>
+      </c>
+      <c r="F20" s="52">
+        <v>0.21567449946463726</v>
+      </c>
+      <c r="G20" s="52">
+        <v>0.16953716943906458</v>
       </c>
       <c r="H20" s="54" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="C21" s="51">
+        <v>0.22772277227722773</v>
+      </c>
+      <c r="D21" s="52">
+        <v>0.1498926626443405</v>
+      </c>
+      <c r="E21" s="52">
+        <v>0.10460975012248896</v>
+      </c>
+      <c r="F21" s="52">
+        <v>0.08101959036116835</v>
+      </c>
+      <c r="G21" s="52">
+        <v>0.06559982005176752</v>
+      </c>
+      <c r="H21" s="54" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="C22" s="59">
+        <v>0.020838048090523337</v>
+      </c>
+      <c r="D22" s="52">
+        <v>0.22649221521704743</v>
+      </c>
+      <c r="E22" s="52">
+        <v>0.40865090641842233</v>
+      </c>
+      <c r="F22" s="52">
+        <v>0.5019717632430317</v>
+      </c>
+      <c r="G22" s="52">
+        <v>0.5640321961663076</v>
+      </c>
+      <c r="H22" s="54" t="s">
         <v>273</v>
       </c>
-      <c r="C21" s="59" t="str">
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="C23" s="60">
+        <v>3</v>
+      </c>
+      <c r="D23" s="60">
+        <v>3</v>
+      </c>
+      <c r="E23" s="60">
+        <v>3</v>
+      </c>
+      <c r="F23" s="60">
+        <v>3</v>
+      </c>
+      <c r="G23" s="60">
+        <v>3</v>
+      </c>
+      <c r="H23" s="54" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="C24" s="61">
+        <v>0.6319081672107103</v>
+      </c>
+      <c r="D24" s="62">
+        <v>10.747650235238861</v>
+      </c>
+      <c r="E24" s="62">
+        <v>28.61956160951256</v>
+      </c>
+      <c r="F24" s="62">
+        <v>46.752155680255555</v>
+      </c>
+      <c r="G24" s="62">
+        <v>66.82825457722186</v>
+      </c>
+      <c r="H24" s="54" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="C25" s="63" t="str">
         <f>IF('5-Year Model'!B58&gt;=0,"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="D21" s="37" t="str">
+      <c r="D25" s="37" t="str">
         <f>IF(AND('5-Year Model'!C58&gt;=0,'5-Year Model'!B58&lt;0),"✓ Break-even","")</f>
         <v>✓ Break-even</v>
       </c>
-      <c r="E21" s="59" t="str">
+      <c r="E25" s="63" t="str">
         <f>IF(AND('5-Year Model'!D58&gt;=0,'5-Year Model'!C58&lt;0),"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="F21" s="59" t="str">
+      <c r="F25" s="63" t="str">
         <f>IF(AND('5-Year Model'!E58&gt;=0,'5-Year Model'!D58&lt;0),"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="G21" s="59" t="str">
+      <c r="G25" s="63" t="str">
         <f>IF(AND('5-Year Model'!F58&gt;=0,'5-Year Model'!E58&lt;0),"✓ Break-even","")</f>
         <v>0</v>
       </c>
-      <c r="H21" s="54" t="s">
+      <c r="H25" s="54" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="27" t="s">
-        <v>274</v>
-      </c>
-      <c r="C22" s="60">
-        <v>0</v>
-      </c>
-      <c r="D22" s="60">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="C26" s="64">
+        <v>0</v>
+      </c>
+      <c r="D26" s="64">
         <v>3</v>
       </c>
-      <c r="E22" s="60">
+      <c r="E26" s="64">
         <v>10</v>
       </c>
-      <c r="F22" s="61">
+      <c r="F26" s="65">
         <v>21</v>
       </c>
-      <c r="G22" s="56">
+      <c r="G26" s="60">
         <v>34</v>
       </c>
-      <c r="H22" s="54" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>277</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12" t="s">
-        <v>279</v>
-      </c>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-    </row>
-    <row r="25" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="62" t="s">
+      <c r="H26" s="54" t="s">
         <v>280</v>
       </c>
-      <c r="C25" s="37" t="s">
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="27" t="s">
+        <v>200</v>
+      </c>
+      <c r="C27" s="64">
+        <v>0</v>
+      </c>
+      <c r="D27" s="60">
+        <v>91</v>
+      </c>
+      <c r="E27" s="60">
+        <v>318</v>
+      </c>
+      <c r="F27" s="60">
+        <v>637</v>
+      </c>
+      <c r="G27" s="60">
+        <v>1030</v>
+      </c>
+      <c r="H27" s="54" t="s">
         <v>281</v>
       </c>
-      <c r="D25" s="63" t="s">
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="E25" s="63"/>
-      <c r="F25" s="64" t="s">
+      <c r="C29" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="G25" s="64"/>
-      <c r="H25" s="64"/>
-    </row>
-    <row r="26" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="62" t="s">
+      <c r="D29" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="C26" s="65" t="s">
+      <c r="E29" s="12"/>
+      <c r="F29" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="66" t="s">
         <v>286</v>
       </c>
-      <c r="E26" s="63"/>
-      <c r="F26" s="64" t="s">
+      <c r="C30" s="37" t="s">
         <v>287</v>
       </c>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-    </row>
-    <row r="27" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B27" s="62" t="s">
+      <c r="D30" s="67" t="s">
         <v>288</v>
       </c>
-      <c r="C27" s="37" t="s">
-        <v>281</v>
-      </c>
-      <c r="D27" s="63" t="s">
+      <c r="E30" s="67"/>
+      <c r="F30" s="68" t="s">
         <v>289</v>
       </c>
-      <c r="E27" s="63"/>
-      <c r="F27" s="64" t="s">
+      <c r="G30" s="68"/>
+      <c r="H30" s="68"/>
+    </row>
+    <row r="31" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="66" t="s">
         <v>290</v>
       </c>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-    </row>
-    <row r="28" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="62" t="s">
+      <c r="C31" s="69" t="s">
         <v>291</v>
       </c>
-      <c r="C28" s="37" t="s">
-        <v>281</v>
-      </c>
-      <c r="D28" s="63" t="s">
+      <c r="D31" s="67" t="s">
         <v>292</v>
       </c>
-      <c r="E28" s="63"/>
-      <c r="F28" s="64" t="s">
+      <c r="E31" s="67"/>
+      <c r="F31" s="68" t="s">
         <v>293</v>
       </c>
-      <c r="G28" s="64"/>
-      <c r="H28" s="64"/>
-    </row>
-    <row r="29" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="62" t="s">
+      <c r="G31" s="68"/>
+      <c r="H31" s="68"/>
+    </row>
+    <row r="32" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="66" t="s">
         <v>294</v>
       </c>
-      <c r="C29" s="37" t="s">
-        <v>281</v>
-      </c>
-      <c r="D29" s="63" t="s">
+      <c r="C32" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D32" s="67" t="s">
         <v>295</v>
       </c>
-      <c r="E29" s="63"/>
-      <c r="F29" s="64" t="s">
+      <c r="E32" s="67"/>
+      <c r="F32" s="68" t="s">
         <v>296</v>
       </c>
-      <c r="G29" s="64"/>
-      <c r="H29" s="64"/>
-    </row>
-    <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="62" t="s">
+      <c r="G32" s="68"/>
+      <c r="H32" s="68"/>
+    </row>
+    <row r="33" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B33" s="66" t="s">
         <v>297</v>
       </c>
-      <c r="C30" s="37" t="s">
-        <v>281</v>
-      </c>
-      <c r="D30" s="63" t="s">
+      <c r="C33" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D33" s="67" t="s">
         <v>298</v>
       </c>
-      <c r="E30" s="63"/>
-      <c r="F30" s="64" t="s">
+      <c r="E33" s="67"/>
+      <c r="F33" s="68" t="s">
         <v>299</v>
       </c>
-      <c r="G30" s="64"/>
-      <c r="H30" s="64"/>
-    </row>
-    <row r="31" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B31" s="62" t="s">
+      <c r="G33" s="68"/>
+      <c r="H33" s="68"/>
+    </row>
+    <row r="34" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B34" s="66" t="s">
         <v>300</v>
       </c>
-      <c r="C31" s="37" t="s">
-        <v>281</v>
-      </c>
-      <c r="D31" s="63" t="s">
+      <c r="C34" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D34" s="67" t="s">
         <v>301</v>
       </c>
-      <c r="E31" s="63"/>
-      <c r="F31" s="64" t="s">
+      <c r="E34" s="67"/>
+      <c r="F34" s="68" t="s">
         <v>302</v>
       </c>
-      <c r="G31" s="64"/>
-      <c r="H31" s="64"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="62" t="s">
+      <c r="G34" s="68"/>
+      <c r="H34" s="68"/>
+    </row>
+    <row r="35" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B35" s="66" t="s">
         <v>303</v>
       </c>
-      <c r="C33" s="27" t="s">
+      <c r="C35" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D35" s="67" t="s">
         <v>304</v>
       </c>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="66" t="s">
+      <c r="E35" s="67"/>
+      <c r="F35" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="G35" s="68"/>
+      <c r="H35" s="68"/>
+    </row>
+    <row r="36" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B36" s="66" t="s">
+        <v>306</v>
+      </c>
+      <c r="C36" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D36" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="E36" s="67"/>
+      <c r="F36" s="68" t="s">
+        <v>308</v>
+      </c>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="66" t="s">
+        <v>309</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="27"/>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="70" t="s">
         <v>155</v>
       </c>
-      <c r="C35" s="66"/>
-      <c r="D35" s="66"/>
-      <c r="E35" s="66"/>
-      <c r="F35" s="66"/>
-      <c r="G35" s="66"/>
-      <c r="H35" s="66"/>
+      <c r="C40" s="70"/>
+      <c r="D40" s="70"/>
+      <c r="E40" s="70"/>
+      <c r="F40" s="70"/>
+      <c r="G40" s="70"/>
+      <c r="H40" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="20">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:H28"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="F29:H29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="F30:H30"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:H31"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="C38:F38"/>
+    <mergeCell ref="B40:H40"/>
   </mergeCells>
   <conditionalFormatting sqref="C12:G12">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -7181,48 +7317,48 @@
       <formula>C15&lt;7000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C16:G16">
+  <conditionalFormatting sqref="C20:G20">
     <cfRule type="expression" dxfId="12" priority="1">
-      <formula>C16&lt;=0.55</formula>
+      <formula>C20&lt;=0.55</formula>
     </cfRule>
     <cfRule type="expression" dxfId="13" priority="2">
-      <formula>C16&lt;=0.65</formula>
+      <formula>C20&lt;=0.65</formula>
     </cfRule>
     <cfRule type="expression" dxfId="14" priority="3">
-      <formula>C16&gt;0.65</formula>
+      <formula>C20&gt;0.65</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C17:G17">
+  <conditionalFormatting sqref="C21:G21">
     <cfRule type="expression" dxfId="15" priority="1">
-      <formula>C17&lt;=0.15</formula>
+      <formula>C21&lt;=0.15</formula>
     </cfRule>
     <cfRule type="expression" dxfId="16" priority="2">
-      <formula>C17&lt;=0.22</formula>
+      <formula>C21&lt;=0.22</formula>
     </cfRule>
     <cfRule type="expression" dxfId="17" priority="3">
-      <formula>C17&gt;0.22</formula>
+      <formula>C21&gt;0.22</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18:G18">
+  <conditionalFormatting sqref="C22:G22">
     <cfRule type="expression" dxfId="18" priority="1">
-      <formula>C18&gt;=0.10</formula>
+      <formula>C22&gt;=0.10</formula>
     </cfRule>
     <cfRule type="expression" dxfId="19" priority="2">
-      <formula>C18&gt;=0</formula>
+      <formula>C22&gt;=0</formula>
     </cfRule>
     <cfRule type="expression" dxfId="20" priority="3">
-      <formula>C18&lt;0</formula>
+      <formula>C22&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C20:G20">
+  <conditionalFormatting sqref="C24:G24">
     <cfRule type="expression" dxfId="21" priority="1">
-      <formula>C20&gt;=1.25</formula>
+      <formula>C24&gt;=1.25</formula>
     </cfRule>
     <cfRule type="expression" dxfId="22" priority="2">
-      <formula>C20&gt;=1</formula>
+      <formula>C24&gt;=1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="23" priority="3">
-      <formula>C20&lt;1</formula>
+      <formula>C24&lt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Task #598: Final underwriting QA fixes + proof pack
Three code fixes in the underwriting guest wizard payload builder:

1. Deferred founder comp: Staffing row now emitted whenever
   founderAnnualCompensation > 0 (not only when founderIsPaidYear1),
   with startYear clamped to [1,5] and deferred note added.

2. Collection rate: perStudentTuition is now multiplied by
   tuitionCollectionRate/100 in the payload builder before sending to
   the engine, so 95% collection → $11,400 effective per-student.

3. Lender readiness founder flag: Distinguishes deferred comp (caution)
   from no comp planned (high severity).

All validations pass: typecheck, 1096 unit tests, 8 e2e smoke, 37 API
tests, 30/30 Excel QA exports, formula results cross-tab, 32/32 smoke
arithmetic.

Proof pack created: docs/UNDERWRITING_GUEST_WIZARD_PROOF_PACK_2026-05-07.md
Verdict: GO
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Formula_Export_Charter_ADA_Grade-Band.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Year 1 Pro Forma'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Decision History'!$A1:$H4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Decision History'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Financial Health'!$A1:$H40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Financial Health'!$A1:$I40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Financial Health'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -38,7 +38,7 @@
     <t>Heritage Academy Charter</t>
   </si>
   <si>
-    <t>Generated May 1, 2026 · nonprofit_501c3</t>
+    <t>Generated May 7, 2026 · nonprofit_501c3</t>
   </si>
   <si>
     <t>Cell Color Legend</t>
@@ -779,7 +779,7 @@
     <t>Heritage Academy Charter — Financial Health Dashboard</t>
   </si>
   <si>
-    <t>Generated May 1, 2026</t>
+    <t>Generated May 7, 2026</t>
   </si>
   <si>
     <t>● Green = healthy</t>
@@ -911,7 +911,7 @@
     <t>The model reaches net income early and sustains strong margins through Year 5.</t>
   </si>
   <si>
-    <t>Monitor enrollment actuals vs. projections in Year 1.</t>
+    <t>Compare your real Year 1 enrollment against this projection as students enroll.</t>
   </si>
   <si>
     <t>Liquidity</t>
@@ -6657,7 +6657,7 @@
     <tabColor rgb="FF328555"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H40"/>
+  <dimension ref="B2:I40"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -6667,7 +6667,7 @@
     <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" ht="30" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>248</v>
       </c>
@@ -6677,8 +6677,9 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="47" t="s">
         <v>249</v>
       </c>
@@ -6688,6 +6689,7 @@
       <c r="F3" s="47"/>
       <c r="G3" s="47"/>
       <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="48" t="s">
@@ -7178,7 +7180,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="29" ht="24" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
         <v>286</v>
       </c>
@@ -7194,8 +7196,9 @@
       </c>
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
-    </row>
-    <row r="30" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I29" s="12"/>
+    </row>
+    <row r="30" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="65" t="s">
         <v>290</v>
       </c>
@@ -7211,8 +7214,9 @@
       </c>
       <c r="G30" s="67"/>
       <c r="H30" s="67"/>
-    </row>
-    <row r="31" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I30" s="67"/>
+    </row>
+    <row r="31" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="65" t="s">
         <v>294</v>
       </c>
@@ -7228,8 +7232,9 @@
       </c>
       <c r="G31" s="67"/>
       <c r="H31" s="67"/>
-    </row>
-    <row r="32" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I31" s="67"/>
+    </row>
+    <row r="32" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="65" t="s">
         <v>297</v>
       </c>
@@ -7245,8 +7250,9 @@
       </c>
       <c r="G32" s="67"/>
       <c r="H32" s="67"/>
-    </row>
-    <row r="33" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I32" s="67"/>
+    </row>
+    <row r="33" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="65" t="s">
         <v>300</v>
       </c>
@@ -7262,8 +7268,9 @@
       </c>
       <c r="G33" s="67"/>
       <c r="H33" s="67"/>
-    </row>
-    <row r="34" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I33" s="67"/>
+    </row>
+    <row r="34" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="65" t="s">
         <v>303</v>
       </c>
@@ -7279,8 +7286,9 @@
       </c>
       <c r="G34" s="67"/>
       <c r="H34" s="67"/>
-    </row>
-    <row r="35" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I34" s="67"/>
+    </row>
+    <row r="35" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="65" t="s">
         <v>306</v>
       </c>
@@ -7296,8 +7304,9 @@
       </c>
       <c r="G35" s="67"/>
       <c r="H35" s="67"/>
-    </row>
-    <row r="36" ht="45" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I35" s="67"/>
+    </row>
+    <row r="36" ht="45" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="65" t="s">
         <v>309</v>
       </c>
@@ -7313,6 +7322,7 @@
       </c>
       <c r="G36" s="67"/>
       <c r="H36" s="67"/>
+      <c r="I36" s="67"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="65" t="s">
@@ -7325,7 +7335,7 @@
       <c r="E38" s="28"/>
       <c r="F38" s="28"/>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="68" t="s">
         <v>155</v>
       </c>
@@ -7335,29 +7345,30 @@
       <c r="F40" s="68"/>
       <c r="G40" s="68"/>
       <c r="H40" s="68"/>
+      <c r="I40" s="68"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="F29:I29"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="F30:I30"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="F31:I31"/>
     <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="F32:I32"/>
     <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="F33:I33"/>
     <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="F34:I34"/>
     <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F35:I35"/>
     <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="F36:I36"/>
     <mergeCell ref="C38:F38"/>
-    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="B40:I40"/>
   </mergeCells>
   <conditionalFormatting sqref="C12:G12">
     <cfRule type="expression" dxfId="0" priority="1">

</xml_diff>